<commit_message>
Subzona de Lanus: se guarda sola con el viaje
R12 = Zona 4, R13 = Zona 17, R16 = Zona 8, R17 = Zona 14. El dato no se
muestra ni se edita: lo pone el sistema al crear o editar el viaje, y sale
en los reportes y en el conteo por localidad.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/server/templates/plantilla_viajes.xlsx
+++ b/server/templates/plantilla_viajes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\AppData\Local\Temp\claude\C--Users-Usuario-Desktop-Claude\9412c732-44f7-4c59-81e4-7e6c39b64ad2\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8335B0D-D619-4911-8F05-05BB88FF713D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F150F398-2F39-4858-AC4F-9B1803461534}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2160" yWindow="2160" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="Viajes" sheetId="1" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Viajes!$A$1:$AC$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Viajes!$A$1:$AD$3</definedName>
   </definedNames>
   <calcPr calcId="0"/>
   <pivotCaches>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="65">
   <si>
     <t>ID viaje</t>
   </si>
@@ -44,6 +44,9 @@
     <t>Zona</t>
   </si>
   <si>
+    <t>Subzona</t>
+  </si>
+  <si>
     <t>Localidad</t>
   </si>
   <si>
@@ -123,6 +126,9 @@
   </si>
   <si>
     <t>LANUS</t>
+  </si>
+  <si>
+    <t>Zona 4</t>
   </si>
   <si>
     <t>SAE</t>
@@ -806,7 +812,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-2B9B-4A27-AC8E-B5CF16EAC395}"/>
+              <c16:uniqueId val="{00000001-4C54-4060-B042-3352E9DCBAFF}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -865,7 +871,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-2B9B-4A27-AC8E-B5CF16EAC395}"/>
+              <c16:uniqueId val="{00000002-4C54-4060-B042-3352E9DCBAFF}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -924,7 +930,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-2B9B-4A27-AC8E-B5CF16EAC395}"/>
+              <c16:uniqueId val="{00000003-4C54-4060-B042-3352E9DCBAFF}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -983,7 +989,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-2B9B-4A27-AC8E-B5CF16EAC395}"/>
+              <c16:uniqueId val="{00000004-4C54-4060-B042-3352E9DCBAFF}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1039,7 +1045,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000005-2B9B-4A27-AC8E-B5CF16EAC395}"/>
+              <c16:uniqueId val="{00000005-4C54-4060-B042-3352E9DCBAFF}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1095,7 +1101,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000006-2B9B-4A27-AC8E-B5CF16EAC395}"/>
+              <c16:uniqueId val="{00000006-4C54-4060-B042-3352E9DCBAFF}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1109,11 +1115,11 @@
         </c:dLbls>
         <c:gapWidth val="219"/>
         <c:overlap val="-27"/>
-        <c:axId val="2121660479"/>
-        <c:axId val="2021911439"/>
+        <c:axId val="1397145696"/>
+        <c:axId val="1394065616"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="2121660479"/>
+        <c:axId val="1397145696"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1156,7 +1162,7 @@
             <a:endParaRPr lang="es-AR"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2021911439"/>
+        <c:crossAx val="1394065616"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1164,7 +1170,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="2021911439"/>
+        <c:axId val="1394065616"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1215,7 +1221,7 @@
             <a:endParaRPr lang="es-AR"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2121660479"/>
+        <c:crossAx val="1397145696"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1849,7 +1855,7 @@
         <xdr:cNvPr id="2" name="Gráfico 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FBE15A94-6EAB-7B40-7BF7-4B8C005E29AC}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{810AA316-6667-4626-BE64-645FC9492116}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1871,11 +1877,11 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Usuario" refreshedDate="46290.601893981482" missingItemsLimit="2" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="3" xr:uid="{A3863CB3-21C4-45C4-9548-D2BAD5E6B29C}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Usuario" refreshedDate="46290.623472685184" missingItemsLimit="2" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="3" xr:uid="{226F4026-52DE-4505-80B0-BEE7E1377794}">
   <cacheSource type="worksheet">
-    <worksheetSource ref="A1:AC5000" sheet="Viajes"/>
+    <worksheetSource ref="A1:AD5000" sheet="Viajes"/>
   </cacheSource>
-  <cacheFields count="29">
+  <cacheFields count="30">
     <cacheField name="ID viaje" numFmtId="0">
       <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="7983" maxValue="7984"/>
     </cacheField>
@@ -1897,6 +1903,9 @@
         <s v="DON ORIONE"/>
         <m/>
       </sharedItems>
+    </cacheField>
+    <cacheField name="Subzona" numFmtId="0">
+      <sharedItems containsBlank="1"/>
     </cacheField>
     <cacheField name="Localidad" numFmtId="0">
       <sharedItems containsBlank="1"/>
@@ -1994,6 +2003,7 @@
     <x v="0"/>
     <s v="R12"/>
     <x v="0"/>
+    <s v="Zona 4"/>
     <s v="LANUS"/>
     <x v="0"/>
     <x v="0"/>
@@ -2025,6 +2035,7 @@
     <x v="0"/>
     <s v="R6"/>
     <x v="1"/>
+    <m/>
     <s v="DON ORIONE"/>
     <x v="0"/>
     <x v="1"/>
@@ -2057,6 +2068,7 @@
     <m/>
     <x v="2"/>
     <m/>
+    <m/>
     <x v="1"/>
     <x v="2"/>
     <m/>
@@ -2085,9 +2097,9 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{27179CAA-B683-46D2-ACC1-BD9FF23586F3}" name="DinamicaViajes" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0" chartFormat="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{51256B52-5966-494D-898B-A9080C5489CF}" name="DinamicaViajes" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0" chartFormat="1">
   <location ref="A7:I13" firstHeaderRow="1" firstDataRow="3" firstDataCol="1" rowPageCount="2" colPageCount="1"/>
-  <pivotFields count="29">
+  <pivotFields count="30">
     <pivotField dataField="1" compact="0" outline="0" showAll="0"/>
     <pivotField compact="0" outline="0" showAll="0"/>
     <pivotField axis="axisPage" compact="0" outline="0" showAll="0">
@@ -2115,6 +2127,7 @@
         </pivotArea>
       </autoSortScope>
     </pivotField>
+    <pivotField compact="0" outline="0" showAll="0"/>
     <pivotField compact="0" outline="0" showAll="0"/>
     <pivotField axis="axisPage" compact="0" outline="0" showAll="0">
       <items count="3">
@@ -2171,7 +2184,7 @@
     </i>
   </rowItems>
   <colFields count="2">
-    <field x="7"/>
+    <field x="8"/>
     <field x="-2"/>
   </colFields>
   <colItems count="8">
@@ -2204,12 +2217,12 @@
     </i>
   </colItems>
   <pageFields count="2">
-    <pageField fld="6" hier="-1"/>
+    <pageField fld="7" hier="-1"/>
     <pageField fld="2" hier="-1"/>
   </pageFields>
   <dataFields count="2">
     <dataField name="Viajes" fld="0" subtotal="count" baseField="0" baseItem="0" numFmtId="3"/>
-    <dataField name="Costo total" fld="26" baseField="0" baseItem="0" numFmtId="168"/>
+    <dataField name="Costo total" fld="27" baseField="0" baseItem="0" numFmtId="168"/>
   </dataFields>
   <chartFormats count="6">
     <chartFormat chart="0" format="0" series="1">
@@ -2218,7 +2231,7 @@
           <reference field="4294967294" count="1" selected="0">
             <x v="0"/>
           </reference>
-          <reference field="7" count="1" selected="0">
+          <reference field="8" count="1" selected="0">
             <x v="0"/>
           </reference>
         </references>
@@ -2230,7 +2243,7 @@
           <reference field="4294967294" count="1" selected="0">
             <x v="1"/>
           </reference>
-          <reference field="7" count="1" selected="0">
+          <reference field="8" count="1" selected="0">
             <x v="0"/>
           </reference>
         </references>
@@ -2242,7 +2255,7 @@
           <reference field="4294967294" count="1" selected="0">
             <x v="0"/>
           </reference>
-          <reference field="7" count="1" selected="0">
+          <reference field="8" count="1" selected="0">
             <x v="1"/>
           </reference>
         </references>
@@ -2254,7 +2267,7 @@
           <reference field="4294967294" count="1" selected="0">
             <x v="1"/>
           </reference>
-          <reference field="7" count="1" selected="0">
+          <reference field="8" count="1" selected="0">
             <x v="1"/>
           </reference>
         </references>
@@ -2266,7 +2279,7 @@
           <reference field="4294967294" count="1" selected="0">
             <x v="0"/>
           </reference>
-          <reference field="7" count="1" selected="0">
+          <reference field="8" count="1" selected="0">
             <x v="2"/>
           </reference>
         </references>
@@ -2278,7 +2291,7 @@
           <reference field="4294967294" count="1" selected="0">
             <x v="1"/>
           </reference>
-          <reference field="7" count="1" selected="0">
+          <reference field="8" count="1" selected="0">
             <x v="2"/>
           </reference>
         </references>
@@ -2581,7 +2594,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B21E597-911C-4246-8AEB-4A51F94C5F6E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C376BBB5-AF8D-42CF-BB7E-DF0F1A55E1A8}">
   <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2593,20 +2606,20 @@
   <sheetData>
     <row r="1" spans="1:9" ht="24.6" x14ac:dyDescent="0.4">
       <c r="A1" s="11" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A4" s="8" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
@@ -2614,16 +2627,16 @@
         <v>2</v>
       </c>
       <c r="B5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A7"/>
       <c r="B7" s="8" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D7"/>
       <c r="E7"/>
@@ -2635,22 +2648,22 @@
     <row r="8" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A8"/>
       <c r="B8" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C8"/>
       <c r="D8" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="E8"/>
       <c r="F8" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="G8"/>
       <c r="H8" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="I8" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
@@ -2658,29 +2671,29 @@
         <v>4</v>
       </c>
       <c r="B9" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C9" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D9" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="E9" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F9" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="G9" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="H9"/>
       <c r="I9"/>
     </row>
     <row r="10" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B10" s="9">
         <v>1</v>
@@ -2701,7 +2714,7 @@
     </row>
     <row r="11" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B11" s="9"/>
       <c r="C11" s="10"/>
@@ -2722,7 +2735,7 @@
     </row>
     <row r="12" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B12" s="9"/>
       <c r="C12" s="10"/>
@@ -2735,7 +2748,7 @@
     </row>
     <row r="13" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B13" s="9">
         <v>1</v>
@@ -2821,31 +2834,31 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AC3"/>
+  <dimension ref="A1:AD3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="6" width="11" customWidth="1"/>
-    <col min="7" max="7" width="19" customWidth="1"/>
-    <col min="8" max="10" width="11" customWidth="1"/>
-    <col min="11" max="13" width="12" customWidth="1"/>
-    <col min="14" max="14" width="11" customWidth="1"/>
-    <col min="15" max="15" width="18" customWidth="1"/>
-    <col min="16" max="16" width="11" customWidth="1"/>
-    <col min="17" max="18" width="13" customWidth="1"/>
-    <col min="19" max="19" width="11" customWidth="1"/>
-    <col min="20" max="20" width="17" customWidth="1"/>
-    <col min="21" max="21" width="18" customWidth="1"/>
-    <col min="22" max="22" width="16" customWidth="1"/>
-    <col min="23" max="23" width="22" customWidth="1"/>
-    <col min="24" max="24" width="20" customWidth="1"/>
-    <col min="25" max="25" width="23" customWidth="1"/>
-    <col min="26" max="26" width="15" customWidth="1"/>
-    <col min="27" max="27" width="11" customWidth="1"/>
-    <col min="28" max="28" width="16" customWidth="1"/>
-    <col min="29" max="29" width="15" customWidth="1"/>
+    <col min="1" max="7" width="11" customWidth="1"/>
+    <col min="8" max="8" width="19" customWidth="1"/>
+    <col min="9" max="11" width="11" customWidth="1"/>
+    <col min="12" max="14" width="12" customWidth="1"/>
+    <col min="15" max="15" width="11" customWidth="1"/>
+    <col min="16" max="16" width="18" customWidth="1"/>
+    <col min="17" max="17" width="11" customWidth="1"/>
+    <col min="18" max="19" width="13" customWidth="1"/>
+    <col min="20" max="20" width="11" customWidth="1"/>
+    <col min="21" max="21" width="17" customWidth="1"/>
+    <col min="22" max="22" width="18" customWidth="1"/>
+    <col min="23" max="23" width="16" customWidth="1"/>
+    <col min="24" max="24" width="22" customWidth="1"/>
+    <col min="25" max="25" width="20" customWidth="1"/>
+    <col min="26" max="26" width="23" customWidth="1"/>
+    <col min="27" max="27" width="15" customWidth="1"/>
+    <col min="28" max="28" width="11" customWidth="1"/>
+    <col min="29" max="29" width="16" customWidth="1"/>
+    <col min="30" max="30" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:30" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2933,8 +2946,11 @@
       <c r="AC1" s="1" t="s">
         <v>28</v>
       </c>
+      <c r="AD1" s="1" t="s">
+        <v>29</v>
+      </c>
     </row>
-    <row r="2" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>7983</v>
       </c>
@@ -2942,82 +2958,85 @@
         <v>46289</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="G2" s="2" t="s">
         <v>32</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="L2" s="2"/>
+        <v>37</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>38</v>
+      </c>
       <c r="M2" s="2"/>
-      <c r="N2" s="2" t="s">
-        <v>37</v>
-      </c>
+      <c r="N2" s="2"/>
       <c r="O2" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="P2" s="2">
+        <v>39</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q2" s="2">
         <v>1</v>
       </c>
-      <c r="Q2" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="R2" s="2"/>
-      <c r="S2" s="2" t="s">
-        <v>40</v>
-      </c>
+      <c r="R2" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="S2" s="2"/>
       <c r="T2" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="U2" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="V2" s="4">
+        <v>43</v>
+      </c>
+      <c r="V2" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="W2" s="4">
         <v>5.5</v>
-      </c>
-      <c r="W2" s="2">
-        <v>12</v>
       </c>
       <c r="X2" s="2">
         <v>12</v>
       </c>
       <c r="Y2" s="2">
+        <v>12</v>
+      </c>
+      <c r="Z2" s="2">
         <v>0</v>
       </c>
-      <c r="Z2" s="5">
+      <c r="AA2" s="5">
         <v>48.2</v>
       </c>
-      <c r="AA2" s="6">
+      <c r="AB2" s="6">
         <v>250000</v>
       </c>
-      <c r="AB2" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="AC2" s="3">
+      <c r="AC2" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="AD2" s="3">
         <v>46295</v>
       </c>
     </row>
-    <row r="3" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:30" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>7984</v>
       </c>
@@ -3025,79 +3044,80 @@
         <v>46289</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>45</v>
-      </c>
+        <v>47</v>
+      </c>
+      <c r="F3" s="2"/>
       <c r="G3" s="2" t="s">
-        <v>32</v>
+        <v>47</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="K3" s="2"/>
+        <v>49</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>50</v>
+      </c>
       <c r="L3" s="2"/>
       <c r="M3" s="2"/>
-      <c r="N3" s="2" t="s">
-        <v>49</v>
-      </c>
+      <c r="N3" s="2"/>
       <c r="O3" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="P3" s="2">
+        <v>51</v>
+      </c>
+      <c r="P3" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q3" s="2">
         <v>1</v>
       </c>
-      <c r="Q3" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="R3" s="2">
+      <c r="R3" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="S3" s="2">
         <v>4</v>
       </c>
-      <c r="S3" s="2" t="s">
-        <v>40</v>
-      </c>
       <c r="T3" s="2" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="U3" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="V3" s="4">
+        <v>53</v>
+      </c>
+      <c r="V3" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="W3" s="4">
         <v>4.47</v>
       </c>
-      <c r="W3" s="2">
+      <c r="X3" s="2">
         <v>10</v>
       </c>
-      <c r="X3" s="2">
+      <c r="Y3" s="2">
         <v>9</v>
       </c>
-      <c r="Y3" s="2">
+      <c r="Z3" s="2">
         <v>1</v>
       </c>
-      <c r="Z3" s="5">
+      <c r="AA3" s="5">
         <v>39</v>
       </c>
-      <c r="AA3" s="6">
+      <c r="AB3" s="6">
         <v>0</v>
       </c>
-      <c r="AB3" s="2"/>
-      <c r="AC3" s="3"/>
+      <c r="AC3" s="2"/>
+      <c r="AD3" s="3"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AC3" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:AD3" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
El export de viajes suma la hoja "Conteo por UN"
Tercera hoja con el conteo de viajes por unidad de negocio, armado con los
MISMOS viajes que se exportan: si filtras por un dia, el analisis es de ese
dia. Sale plano (una fila por categoria, los 12 meses y el total) para poder
filtrarlo y pivotearlo en Excel.

Lo calcula la web con las mismas tablas de la pantalla y el servidor solo lo
escribe, asi no hay dos logicas que puedan dar numeros distintos.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/server/templates/plantilla_viajes.xlsx
+++ b/server/templates/plantilla_viajes.xlsx
@@ -5,29 +5,31 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\AppData\Local\Temp\claude\C--Users-Usuario-Desktop-Claude\9412c732-44f7-4c59-81e4-7e6c39b64ad2\scratchpad\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\AppData\Local\Temp\claude\C--Users-Usuario-Desktop-Claude\1ce4d530-0c0c-4c21-82f2-074c99f26bbd\scratchpad\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F150F398-2F39-4858-AC4F-9B1803461534}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99097B4D-F268-4767-A948-921F60BE5FBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2160" yWindow="2160" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Resumen" sheetId="2" r:id="rId1"/>
+    <sheet name="Resumen" sheetId="3" r:id="rId1"/>
     <sheet name="Viajes" sheetId="1" r:id="rId2"/>
+    <sheet name="Conteo por UN" sheetId="2" r:id="rId3"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Conteo por UN'!$A$1:$P$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Viajes!$A$1:$AD$3</definedName>
   </definedNames>
   <calcPr calcId="0"/>
   <pivotCaches>
-    <pivotCache cacheId="8" r:id="rId3"/>
+    <pivotCache cacheId="16" r:id="rId4"/>
   </pivotCaches>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="83">
   <si>
     <t>ID viaje</t>
   </si>
@@ -192,6 +194,60 @@
   </si>
   <si>
     <t>10:02</t>
+  </si>
+  <si>
+    <t>Region</t>
+  </si>
+  <si>
+    <t>Categoria</t>
+  </si>
+  <si>
+    <t>Ene</t>
+  </si>
+  <si>
+    <t>Feb</t>
+  </si>
+  <si>
+    <t>Mar</t>
+  </si>
+  <si>
+    <t>Abr</t>
+  </si>
+  <si>
+    <t>May</t>
+  </si>
+  <si>
+    <t>Jun</t>
+  </si>
+  <si>
+    <t>Jul</t>
+  </si>
+  <si>
+    <t>Ago</t>
+  </si>
+  <si>
+    <t>Sep</t>
+  </si>
+  <si>
+    <t>Oct</t>
+  </si>
+  <si>
+    <t>Nov</t>
+  </si>
+  <si>
+    <t>Dic</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>SAE BROWN</t>
+  </si>
+  <si>
+    <t>Longchamps</t>
+  </si>
+  <si>
+    <t>SAE LANUS</t>
   </si>
   <si>
     <t>(en blanco)</t>
@@ -377,7 +433,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr lang="es-AR"/>
+              <a:rPr lang="en-US"/>
               <a:t>Viajes por zona</a:t>
             </a:r>
           </a:p>
@@ -812,7 +868,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-4C54-4060-B042-3352E9DCBAFF}"/>
+              <c16:uniqueId val="{00000001-035A-49A7-BC90-68F65052A38C}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -871,7 +927,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-4C54-4060-B042-3352E9DCBAFF}"/>
+              <c16:uniqueId val="{00000002-035A-49A7-BC90-68F65052A38C}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -930,7 +986,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-4C54-4060-B042-3352E9DCBAFF}"/>
+              <c16:uniqueId val="{00000003-035A-49A7-BC90-68F65052A38C}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -989,7 +1045,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000004-4C54-4060-B042-3352E9DCBAFF}"/>
+              <c16:uniqueId val="{00000004-035A-49A7-BC90-68F65052A38C}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1045,7 +1101,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000005-4C54-4060-B042-3352E9DCBAFF}"/>
+              <c16:uniqueId val="{00000005-035A-49A7-BC90-68F65052A38C}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1101,7 +1157,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000006-4C54-4060-B042-3352E9DCBAFF}"/>
+              <c16:uniqueId val="{00000006-035A-49A7-BC90-68F65052A38C}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1115,11 +1171,11 @@
         </c:dLbls>
         <c:gapWidth val="219"/>
         <c:overlap val="-27"/>
-        <c:axId val="1397145696"/>
-        <c:axId val="1394065616"/>
+        <c:axId val="1303079184"/>
+        <c:axId val="79736655"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1397145696"/>
+        <c:axId val="1303079184"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1162,7 +1218,7 @@
             <a:endParaRPr lang="es-AR"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1394065616"/>
+        <c:crossAx val="79736655"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1170,7 +1226,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1394065616"/>
+        <c:axId val="79736655"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1221,7 +1277,7 @@
             <a:endParaRPr lang="es-AR"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1397145696"/>
+        <c:crossAx val="1303079184"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1855,7 +1911,7 @@
         <xdr:cNvPr id="2" name="Gráfico 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{810AA316-6667-4626-BE64-645FC9492116}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B6700B92-286C-2DD3-AA32-AA428508B0B8}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1877,7 +1933,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Usuario" refreshedDate="46290.623472685184" missingItemsLimit="2" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="3" xr:uid="{226F4026-52DE-4505-80B0-BEE7E1377794}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Usuario" refreshedDate="46292.736203356479" missingItemsLimit="2" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="3" xr:uid="{C8E61F73-F38D-44AD-9777-2EE45D8FECB0}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A1:AD5000" sheet="Viajes"/>
   </cacheSource>
@@ -2097,7 +2153,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{51256B52-5966-494D-898B-A9080C5489CF}" name="DinamicaViajes" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0" chartFormat="1">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{5B51A289-81D0-402F-AAD0-78A46F7454B7}" name="DinamicaViajes" cacheId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" compact="0" compactData="0" multipleFieldFilters="0" chartFormat="1">
   <location ref="A7:I13" firstHeaderRow="1" firstDataRow="3" firstDataCol="1" rowPageCount="2" colPageCount="1"/>
   <pivotFields count="30">
     <pivotField dataField="1" compact="0" outline="0" showAll="0"/>
@@ -2594,7 +2650,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C376BBB5-AF8D-42CF-BB7E-DF0F1A55E1A8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{918E3099-D38D-47D9-A7AA-126E9DCE5B39}">
   <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2606,12 +2662,12 @@
   <sheetData>
     <row r="1" spans="1:9" ht="24.6" x14ac:dyDescent="0.4">
       <c r="A1" s="11" t="s">
-        <v>63</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>64</v>
+        <v>82</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
@@ -2619,7 +2675,7 @@
         <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
@@ -2627,7 +2683,7 @@
         <v>2</v>
       </c>
       <c r="B5" t="s">
-        <v>57</v>
+        <v>75</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
@@ -2636,7 +2692,7 @@
         <v>8</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>62</v>
+        <v>80</v>
       </c>
       <c r="D7"/>
       <c r="E7"/>
@@ -2656,14 +2712,14 @@
       </c>
       <c r="E8"/>
       <c r="F8" t="s">
-        <v>55</v>
+        <v>73</v>
       </c>
       <c r="G8"/>
       <c r="H8" t="s">
-        <v>59</v>
+        <v>77</v>
       </c>
       <c r="I8" t="s">
-        <v>60</v>
+        <v>78</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
@@ -2671,22 +2727,22 @@
         <v>4</v>
       </c>
       <c r="B9" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="C9" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="D9" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="E9" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="F9" t="s">
-        <v>58</v>
+        <v>76</v>
       </c>
       <c r="G9" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="H9"/>
       <c r="I9"/>
@@ -2735,7 +2791,7 @@
     </row>
     <row r="12" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>55</v>
+        <v>73</v>
       </c>
       <c r="B12" s="9"/>
       <c r="C12" s="10"/>
@@ -2748,7 +2804,7 @@
     </row>
     <row r="13" spans="1:9" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="B13" s="9">
         <v>1</v>
@@ -2828,7 +2884,8 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId2"/>
+  <pageSetup paperSize="267" orientation="portrait" horizontalDpi="203" verticalDpi="203" r:id="rId2"/>
+  <drawing r:id="rId3"/>
 </worksheet>
 </file>
 
@@ -3120,4 +3177,172 @@
   <autoFilter ref="A1:AD3" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:P3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="26" customWidth="1"/>
+    <col min="4" max="15" width="7" customWidth="1"/>
+    <col min="16" max="16" width="10" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="D2" s="2">
+        <v>0</v>
+      </c>
+      <c r="E2" s="2">
+        <v>0</v>
+      </c>
+      <c r="F2" s="2">
+        <v>6</v>
+      </c>
+      <c r="G2" s="2">
+        <v>1</v>
+      </c>
+      <c r="H2" s="2">
+        <v>13</v>
+      </c>
+      <c r="I2" s="2">
+        <v>11</v>
+      </c>
+      <c r="J2" s="2">
+        <v>7</v>
+      </c>
+      <c r="K2" s="2">
+        <v>23</v>
+      </c>
+      <c r="L2" s="2">
+        <v>42</v>
+      </c>
+      <c r="M2" s="2">
+        <v>0</v>
+      </c>
+      <c r="N2" s="2">
+        <v>0</v>
+      </c>
+      <c r="O2" s="2">
+        <v>0</v>
+      </c>
+      <c r="P2" s="2">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="D3" s="2">
+        <v>0</v>
+      </c>
+      <c r="E3" s="2">
+        <v>0</v>
+      </c>
+      <c r="F3" s="2">
+        <v>0</v>
+      </c>
+      <c r="G3" s="2">
+        <v>0</v>
+      </c>
+      <c r="H3" s="2">
+        <v>5</v>
+      </c>
+      <c r="I3" s="2">
+        <v>9</v>
+      </c>
+      <c r="J3" s="2">
+        <v>12</v>
+      </c>
+      <c r="K3" s="2">
+        <v>30</v>
+      </c>
+      <c r="L3" s="2">
+        <v>39</v>
+      </c>
+      <c r="M3" s="2">
+        <v>0</v>
+      </c>
+      <c r="N3" s="2">
+        <v>0</v>
+      </c>
+      <c r="O3" s="2">
+        <v>0</v>
+      </c>
+      <c r="P3" s="2">
+        <v>95</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:P3" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
El export marca a que categoria del conteo pertenece cada viaje
Dos columnas nuevas en la hoja Viajes: "Region UN" y "Categoria UN", con la
misma clasificacion del cuadro. Asi se puede filtrar el detalle por categoria,
y en la dinamica del Resumen se puede hacer doble clic sobre un numero para
que Excel arme la lista de esos viajes.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/server/templates/plantilla_viajes.xlsx
+++ b/server/templates/plantilla_viajes.xlsx
@@ -11,11 +11,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conteo por UN" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Viajes'!$A$1:$AD$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Viajes'!$A$1:$AF$3</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
   <pivotCaches>
-    <pivotCache xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cacheId="16" r:id="rId4"/>
+    <pivotCache xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cacheId="8" r:id="rId4"/>
   </pivotCaches>
 </workbook>
 </file>
@@ -290,7 +290,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:rPr lang="en-US"/>
+              <a:rPr lang="es-AR"/>
               <a:t>Viajes por zona</a:t>
             </a:r>
           </a:p>
@@ -1030,11 +1030,11 @@
         </dLbls>
         <gapWidth val="219"/>
         <overlap val="-27"/>
-        <axId val="42854912"/>
-        <axId val="86611856"/>
+        <axId val="35631663"/>
+        <axId val="1640146991"/>
       </barChart>
       <catAx>
-        <axId val="42854912"/>
+        <axId val="35631663"/>
         <scaling>
           <orientation val="minMax"/>
         </scaling>
@@ -1080,7 +1080,7 @@
             <a:endParaRPr lang="es-AR"/>
           </a:p>
         </txPr>
-        <crossAx val="86611856"/>
+        <crossAx val="1640146991"/>
         <crosses val="autoZero"/>
         <auto val="1"/>
         <lblAlgn val="ctr"/>
@@ -1088,7 +1088,7 @@
         <noMultiLvlLbl val="0"/>
       </catAx>
       <valAx>
-        <axId val="86611856"/>
+        <axId val="1640146991"/>
         <scaling>
           <orientation val="minMax"/>
         </scaling>
@@ -1142,7 +1142,7 @@
             <a:endParaRPr lang="es-AR"/>
           </a:p>
         </txPr>
-        <crossAx val="42854912"/>
+        <crossAx val="35631663"/>
         <crosses val="autoZero"/>
         <crossBetween val="between"/>
       </valAx>
@@ -1201,11 +1201,11 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" refreshOnLoad="1" refreshedBy="Usuario" refreshedDate="46292.74196203703" missingItemsLimit="2" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="3" r:id="rId1">
+<pivotCacheDefinition xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" refreshOnLoad="1" refreshedBy="Usuario" refreshedDate="46292.74943113426" missingItemsLimit="2" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="3" r:id="rId1">
   <cacheSource type="worksheet">
-    <worksheetSource ref="A1:AD5000" sheet="Viajes"/>
+    <worksheetSource ref="A1:AF5000" sheet="Viajes"/>
   </cacheSource>
-  <cacheFields count="30">
+  <cacheFields count="32">
     <cacheField name="ID viaje" uniqueList="1" numFmtId="0" sqlType="0" hierarchy="0" level="0" databaseField="1">
       <sharedItems count="0" containsBlank="1" containsInteger="1" containsNumber="1" containsString="0" minValue="7983" maxValue="7984"/>
     </cacheField>
@@ -1229,6 +1229,12 @@
       </sharedItems>
     </cacheField>
     <cacheField name="Subzona" uniqueList="1" numFmtId="0" sqlType="0" hierarchy="0" level="0" databaseField="1">
+      <sharedItems count="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Region UN" uniqueList="1" numFmtId="0" sqlType="0" hierarchy="0" level="0" databaseField="1">
+      <sharedItems count="0" containsBlank="1"/>
+    </cacheField>
+    <cacheField name="Categoria UN" uniqueList="1" numFmtId="0" sqlType="0" hierarchy="0" level="0" databaseField="1">
       <sharedItems count="0" containsBlank="1"/>
     </cacheField>
     <cacheField name="Localidad" uniqueList="1" numFmtId="0" sqlType="0" hierarchy="0" level="0" databaseField="1">
@@ -1322,6 +1328,8 @@
     <x v="0"/>
     <s v="R12"/>
     <x v="0"/>
+    <s v="Zona 4"/>
+    <s v="SAE LANUS"/>
     <s v="Zona 4"/>
     <s v="LANUS"/>
     <x v="0"/>
@@ -1355,6 +1363,8 @@
     <s v="R6"/>
     <x v="1"/>
     <m/>
+    <s v="SAE BROWN"/>
+    <s v="Don Orione"/>
     <s v="DON ORIONE"/>
     <x v="0"/>
     <x v="1"/>
@@ -1388,6 +1398,8 @@
     <x v="2"/>
     <m/>
     <m/>
+    <m/>
+    <m/>
     <x v="1"/>
     <x v="2"/>
     <m/>
@@ -1416,9 +1428,9 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="DinamicaViajes" cacheId="16" dataOnRows="0" dataCaption="Valores" showError="0" showMissing="1" updatedVersion="8" minRefreshableVersion="3" asteriskTotals="0" showItems="1" editData="0" disableFieldList="0" showCalcMbrs="1" visualTotals="1" showMultipleLabel="1" showDataDropDown="1" showDrill="1" printDrill="0" showMemberPropertyTips="1" showDataTips="1" enableWizard="1" enableDrill="1" enableFieldProperties="1" preserveFormatting="1" useAutoFormatting="1" pageWrap="0" pageOverThenDown="0" subtotalHiddenItems="0" rowGrandTotals="1" colGrandTotals="1" fieldPrintTitles="0" itemPrintTitles="1" mergeItem="0" showDropZones="1" createdVersion="8" indent="0" showEmptyRow="0" showEmptyCol="0" showHeaders="1" compact="0" outline="0" outlineData="0" compactData="0" published="0" gridDropZones="0" immersive="1" multipleFieldFilters="0" chartFormat="1" fieldListSortAscending="0" mdxSubqueries="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" r:id="rId1">
+<pivotTableDefinition xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="DinamicaViajes" cacheId="8" dataOnRows="0" dataCaption="Valores" showError="0" showMissing="1" updatedVersion="8" minRefreshableVersion="3" asteriskTotals="0" showItems="1" editData="0" disableFieldList="0" showCalcMbrs="1" visualTotals="1" showMultipleLabel="1" showDataDropDown="1" showDrill="1" printDrill="0" showMemberPropertyTips="1" showDataTips="1" enableWizard="1" enableDrill="1" enableFieldProperties="1" preserveFormatting="1" useAutoFormatting="1" pageWrap="0" pageOverThenDown="0" subtotalHiddenItems="0" rowGrandTotals="1" colGrandTotals="1" fieldPrintTitles="0" itemPrintTitles="1" mergeItem="0" showDropZones="1" createdVersion="8" indent="0" showEmptyRow="0" showEmptyCol="0" showHeaders="1" compact="0" outline="0" outlineData="0" compactData="0" published="0" gridDropZones="0" immersive="1" multipleFieldFilters="0" chartFormat="1" fieldListSortAscending="0" mdxSubqueries="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" r:id="rId1">
   <location ref="A7:I13" firstHeaderRow="1" firstDataRow="3" firstDataCol="1" rowPageCount="2" colPageCount="1"/>
-  <pivotFields count="30">
+  <pivotFields count="32">
     <pivotField dataField="1" showDropDowns="1" compact="0" outline="0" subtotalTop="1" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" itemPageCount="10" sortType="manual" defaultSubtotal="1"/>
     <pivotField showDropDowns="1" compact="0" outline="0" subtotalTop="1" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" itemPageCount="10" sortType="manual" defaultSubtotal="1"/>
     <pivotField axis="axisPage" showDropDowns="1" compact="0" outline="0" subtotalTop="1" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" itemPageCount="10" sortType="manual" defaultSubtotal="1">
@@ -1446,6 +1458,8 @@
         </pivotArea>
       </autoSortScope>
     </pivotField>
+    <pivotField showDropDowns="1" compact="0" outline="0" subtotalTop="1" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" itemPageCount="10" sortType="manual" defaultSubtotal="1"/>
+    <pivotField showDropDowns="1" compact="0" outline="0" subtotalTop="1" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" itemPageCount="10" sortType="manual" defaultSubtotal="1"/>
     <pivotField showDropDowns="1" compact="0" outline="0" subtotalTop="1" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" itemPageCount="10" sortType="manual" defaultSubtotal="1"/>
     <pivotField showDropDowns="1" compact="0" outline="0" subtotalTop="1" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" itemPageCount="10" sortType="manual" defaultSubtotal="1"/>
     <pivotField axis="axisPage" showDropDowns="1" compact="0" outline="0" subtotalTop="1" dragToRow="1" dragToCol="1" dragToPage="1" dragToData="1" dragOff="1" showAll="0" topAutoShow="1" itemPageCount="10" sortType="manual" defaultSubtotal="1">
@@ -1503,7 +1517,7 @@
     </i>
   </rowItems>
   <colFields count="2">
-    <field x="8"/>
+    <field x="10"/>
     <field x="-2"/>
   </colFields>
   <colItems count="8">
@@ -1536,12 +1550,12 @@
     </i>
   </colItems>
   <pageFields count="2">
-    <pageField fld="7" hier="-1"/>
+    <pageField fld="9" hier="-1"/>
     <pageField fld="2" hier="-1"/>
   </pageFields>
   <dataFields count="2">
     <dataField name="Viajes" fld="0" subtotal="count" showDataAs="normal" baseField="0" baseItem="0" numFmtId="3"/>
-    <dataField name="Costo total" fld="27" subtotal="sum" showDataAs="normal" baseField="0" baseItem="0" numFmtId="168"/>
+    <dataField name="Costo total" fld="29" subtotal="sum" showDataAs="normal" baseField="0" baseItem="0" numFmtId="168"/>
   </dataFields>
   <chartFormats count="6">
     <chartFormat chart="0" format="0" series="1">
@@ -1550,7 +1564,7 @@
           <reference field="4294967294" selected="0">
             <x v="0"/>
           </reference>
-          <reference field="8" selected="0">
+          <reference field="10" selected="0">
             <x v="0"/>
           </reference>
         </references>
@@ -1562,7 +1576,7 @@
           <reference field="4294967294" selected="0">
             <x v="1"/>
           </reference>
-          <reference field="8" selected="0">
+          <reference field="10" selected="0">
             <x v="0"/>
           </reference>
         </references>
@@ -1574,7 +1588,7 @@
           <reference field="4294967294" selected="0">
             <x v="0"/>
           </reference>
-          <reference field="8" selected="0">
+          <reference field="10" selected="0">
             <x v="1"/>
           </reference>
         </references>
@@ -1586,7 +1600,7 @@
           <reference field="4294967294" selected="0">
             <x v="1"/>
           </reference>
-          <reference field="8" selected="0">
+          <reference field="10" selected="0">
             <x v="1"/>
           </reference>
         </references>
@@ -1598,7 +1612,7 @@
           <reference field="4294967294" selected="0">
             <x v="0"/>
           </reference>
-          <reference field="8" selected="0">
+          <reference field="10" selected="0">
             <x v="2"/>
           </reference>
         </references>
@@ -1610,7 +1624,7 @@
           <reference field="4294967294" selected="0">
             <x v="1"/>
           </reference>
-          <reference field="8" selected="0">
+          <reference field="10" selected="0">
             <x v="2"/>
           </reference>
         </references>
@@ -2144,28 +2158,30 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD3"/>
+  <dimension ref="A1:AF3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="7"/>
-    <col width="19" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="11"/>
-    <col width="12" customWidth="1" min="12" max="14"/>
-    <col width="11" customWidth="1" min="15" max="15"/>
-    <col width="18" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="13"/>
+    <col width="12" customWidth="1" min="14" max="16"/>
     <col width="11" customWidth="1" min="17" max="17"/>
-    <col width="13" customWidth="1" min="18" max="19"/>
-    <col width="11" customWidth="1" min="20" max="20"/>
-    <col width="17" customWidth="1" min="21" max="21"/>
-    <col width="18" customWidth="1" min="22" max="22"/>
-    <col width="16" customWidth="1" min="23" max="23"/>
-    <col width="22" customWidth="1" min="24" max="24"/>
-    <col width="20" customWidth="1" min="25" max="25"/>
-    <col width="23" customWidth="1" min="26" max="26"/>
-    <col width="15" customWidth="1" min="27" max="27"/>
-    <col width="11" customWidth="1" min="28" max="28"/>
-    <col width="16" customWidth="1" min="29" max="29"/>
-    <col width="15" customWidth="1" min="30" max="30"/>
+    <col width="18" customWidth="1" min="18" max="18"/>
+    <col width="11" customWidth="1" min="19" max="19"/>
+    <col width="13" customWidth="1" min="20" max="21"/>
+    <col width="11" customWidth="1" min="22" max="22"/>
+    <col width="17" customWidth="1" min="23" max="23"/>
+    <col width="18" customWidth="1" min="24" max="24"/>
+    <col width="16" customWidth="1" min="25" max="25"/>
+    <col width="22" customWidth="1" min="26" max="26"/>
+    <col width="20" customWidth="1" min="27" max="27"/>
+    <col width="23" customWidth="1" min="28" max="28"/>
+    <col width="15" customWidth="1" min="29" max="29"/>
+    <col width="11" customWidth="1" min="30" max="30"/>
+    <col width="16" customWidth="1" min="31" max="31"/>
+    <col width="15" customWidth="1" min="32" max="32"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -2201,120 +2217,130 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Region UN</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Categoria UN</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>Localidad</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Unidad de negocio</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Contrato</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Proveedor</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Chofer</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Auxiliar 1</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Auxiliar 2</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Auxiliar 3</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Patente</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Tipo de vehiculo</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Vuelta</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Refrigerado</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Temperatura</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Salida deposito</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Llegada deposito</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Duracion horas</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Paradas planificadas</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>Paradas entregadas</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Paradas no entregadas</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Km recorridos</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Costo</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>Estado de pago</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>Fecha de pago</t>
         </is>
@@ -2349,94 +2375,104 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
+          <t>SAE LANUS</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Zona 4</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
           <t>LANUS</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>SAE</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>Tercerizado</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
         <is>
           <t>EXTERNO</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>CLAUDIO SALINA</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>DENIS RODRIGUEZ</t>
         </is>
       </c>
-      <c r="M2" s="2" t="n"/>
-      <c r="N2" s="2" t="n"/>
-      <c r="O2" s="2" t="inlineStr">
+      <c r="O2" s="2" t="n"/>
+      <c r="P2" s="2" t="n"/>
+      <c r="Q2" s="2" t="inlineStr">
         <is>
           <t>AA233TQ</t>
         </is>
       </c>
-      <c r="P2" s="2" t="inlineStr">
+      <c r="R2" s="2" t="inlineStr">
         <is>
           <t>VANS</t>
         </is>
       </c>
-      <c r="Q2" s="2" t="n">
+      <c r="S2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="R2" s="2" t="inlineStr">
+      <c r="T2" s="2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="S2" s="2" t="n"/>
-      <c r="T2" s="2" t="inlineStr">
+      <c r="U2" s="2" t="n"/>
+      <c r="V2" s="2" t="inlineStr">
         <is>
           <t>Cerrado</t>
         </is>
       </c>
-      <c r="U2" s="2" t="inlineStr">
+      <c r="W2" s="2" t="inlineStr">
         <is>
           <t>06:10</t>
         </is>
       </c>
-      <c r="V2" s="2" t="inlineStr">
+      <c r="X2" s="2" t="inlineStr">
         <is>
           <t>11:40</t>
         </is>
       </c>
-      <c r="W2" s="4" t="n">
+      <c r="Y2" s="4" t="n">
         <v>5.5</v>
       </c>
-      <c r="X2" s="2" t="n">
+      <c r="Z2" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="Y2" s="2" t="n">
+      <c r="AA2" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="Z2" s="2" t="n">
+      <c r="AB2" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AA2" s="15" t="n">
+      <c r="AC2" s="15" t="n">
         <v>48.2</v>
       </c>
-      <c r="AB2" s="6" t="n">
+      <c r="AD2" s="6" t="n">
         <v>250000</v>
       </c>
-      <c r="AC2" s="2" t="inlineStr">
+      <c r="AE2" s="2" t="inlineStr">
         <is>
           <t>Pagado</t>
         </is>
       </c>
-      <c r="AD2" s="14" t="n">
+      <c r="AF2" s="14" t="n">
         <v>46295</v>
       </c>
     </row>
@@ -2465,91 +2501,101 @@
       <c r="F3" s="2" t="n"/>
       <c r="G3" s="2" t="inlineStr">
         <is>
+          <t>SAE BROWN</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Don Orione</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
           <t>DON ORIONE</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
         <is>
           <t>SAE</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>Propio</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
         <is>
           <t>R14 LOG</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>DIEGO GUIDA</t>
         </is>
       </c>
-      <c r="L3" s="2" t="n"/>
-      <c r="M3" s="2" t="n"/>
       <c r="N3" s="2" t="n"/>
-      <c r="O3" s="2" t="inlineStr">
+      <c r="O3" s="2" t="n"/>
+      <c r="P3" s="2" t="n"/>
+      <c r="Q3" s="2" t="inlineStr">
         <is>
           <t>AB069DL</t>
         </is>
       </c>
-      <c r="P3" s="2" t="inlineStr">
+      <c r="R3" s="2" t="inlineStr">
         <is>
           <t>VANS</t>
         </is>
       </c>
-      <c r="Q3" s="2" t="n">
+      <c r="S3" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="R3" s="2" t="inlineStr">
+      <c r="T3" s="2" t="inlineStr">
         <is>
           <t>Si</t>
         </is>
       </c>
-      <c r="S3" s="2" t="n">
+      <c r="U3" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="T3" s="2" t="inlineStr">
+      <c r="V3" s="2" t="inlineStr">
         <is>
           <t>Cerrado</t>
         </is>
       </c>
-      <c r="U3" s="2" t="inlineStr">
+      <c r="W3" s="2" t="inlineStr">
         <is>
           <t>05:34</t>
         </is>
       </c>
-      <c r="V3" s="2" t="inlineStr">
+      <c r="X3" s="2" t="inlineStr">
         <is>
           <t>10:02</t>
         </is>
       </c>
-      <c r="W3" s="4" t="n">
+      <c r="Y3" s="4" t="n">
         <v>4.47</v>
       </c>
-      <c r="X3" s="2" t="n">
+      <c r="Z3" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="Y3" s="2" t="n">
+      <c r="AA3" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="Z3" s="2" t="n">
+      <c r="AB3" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AA3" s="15" t="n">
+      <c r="AC3" s="15" t="n">
         <v>39</v>
       </c>
-      <c r="AB3" s="6" t="n">
+      <c r="AD3" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="AC3" s="2" t="n"/>
-      <c r="AD3" s="14" t="n"/>
+      <c r="AE3" s="2" t="n"/>
+      <c r="AF3" s="14" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AD3"/>
+  <autoFilter ref="A1:AF3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Renombrar: lo que llamabamos Zona es la Localidad, y Localidad es el Partido
Cambian los rotulos en toda la interfaz, los encabezados de los exports y el
reporte semanal. Los nombres internos de la base no se tocan (trip.zone sigue
siendo zone) y las fichas de las escuelas quedan igual: ya distinguian bien
Localidad de Partido.

La columna "Localidad" que traia el viaje era una copia de la zona y estaba
vacia: se reemplaza por Partido, que sale de la tabla de equivalencias.
El import sigue aceptando planillas viejas con la columna "Zona".

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/server/templates/plantilla_viajes.xlsx
+++ b/server/templates/plantilla_viajes.xlsx
@@ -291,7 +291,7 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="es-AR"/>
-              <a:t>Viajes por zona</a:t>
+              <a:t>Viajes por localidad</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -1030,11 +1030,11 @@
         </dLbls>
         <gapWidth val="219"/>
         <overlap val="-27"/>
-        <axId val="35631663"/>
-        <axId val="1640146991"/>
+        <axId val="1489714063"/>
+        <axId val="1486438927"/>
       </barChart>
       <catAx>
-        <axId val="35631663"/>
+        <axId val="1489714063"/>
         <scaling>
           <orientation val="minMax"/>
         </scaling>
@@ -1080,7 +1080,7 @@
             <a:endParaRPr lang="es-AR"/>
           </a:p>
         </txPr>
-        <crossAx val="1640146991"/>
+        <crossAx val="1486438927"/>
         <crosses val="autoZero"/>
         <auto val="1"/>
         <lblAlgn val="ctr"/>
@@ -1088,7 +1088,7 @@
         <noMultiLvlLbl val="0"/>
       </catAx>
       <valAx>
-        <axId val="1640146991"/>
+        <axId val="1486438927"/>
         <scaling>
           <orientation val="minMax"/>
         </scaling>
@@ -1142,7 +1142,7 @@
             <a:endParaRPr lang="es-AR"/>
           </a:p>
         </txPr>
-        <crossAx val="35631663"/>
+        <crossAx val="1489714063"/>
         <crosses val="autoZero"/>
         <crossBetween val="between"/>
       </valAx>
@@ -1201,7 +1201,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" refreshOnLoad="1" refreshedBy="Usuario" refreshedDate="46292.74943113426" missingItemsLimit="2" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="3" r:id="rId1">
+<pivotCacheDefinition xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" refreshOnLoad="1" refreshedBy="Usuario" refreshedDate="46292.95958495371" missingItemsLimit="2" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="3" r:id="rId1">
   <cacheSource type="worksheet">
     <worksheetSource ref="A1:AF5000" sheet="Viajes"/>
   </cacheSource>
@@ -1221,13 +1221,16 @@
     <cacheField name="Reparto" uniqueList="1" numFmtId="0" sqlType="0" hierarchy="0" level="0" databaseField="1">
       <sharedItems count="0" containsBlank="1"/>
     </cacheField>
-    <cacheField name="Zona" uniqueList="1" numFmtId="0" sqlType="0" hierarchy="0" level="0" databaseField="1">
+    <cacheField name="Localidad" uniqueList="1" numFmtId="0" sqlType="0" hierarchy="0" level="0" databaseField="1">
       <sharedItems count="3" containsBlank="1">
         <s v="LANUS"/>
         <s v="DON ORIONE"/>
         <m/>
       </sharedItems>
     </cacheField>
+    <cacheField name="Partido" uniqueList="1" numFmtId="0" sqlType="0" hierarchy="0" level="0" databaseField="1">
+      <sharedItems count="0" containsBlank="1"/>
+    </cacheField>
     <cacheField name="Subzona" uniqueList="1" numFmtId="0" sqlType="0" hierarchy="0" level="0" databaseField="1">
       <sharedItems count="0" containsBlank="1"/>
     </cacheField>
@@ -1235,9 +1238,6 @@
       <sharedItems count="0" containsBlank="1"/>
     </cacheField>
     <cacheField name="Categoria UN" uniqueList="1" numFmtId="0" sqlType="0" hierarchy="0" level="0" databaseField="1">
-      <sharedItems count="0" containsBlank="1"/>
-    </cacheField>
-    <cacheField name="Localidad" uniqueList="1" numFmtId="0" sqlType="0" hierarchy="0" level="0" databaseField="1">
       <sharedItems count="0" containsBlank="1"/>
     </cacheField>
     <cacheField name="Unidad de negocio" uniqueList="1" numFmtId="0" sqlType="0" hierarchy="0" level="0" databaseField="1">
@@ -1328,10 +1328,10 @@
     <x v="0"/>
     <s v="R12"/>
     <x v="0"/>
+    <s v="Lanus"/>
     <s v="Zona 4"/>
     <s v="SAE LANUS"/>
     <s v="Zona 4"/>
-    <s v="LANUS"/>
     <x v="0"/>
     <x v="0"/>
     <s v="EXTERNO"/>
@@ -1362,10 +1362,10 @@
     <x v="0"/>
     <s v="R6"/>
     <x v="1"/>
+    <s v="Almirante Brown"/>
     <m/>
     <s v="SAE BROWN"/>
     <s v="Don Orione"/>
-    <s v="DON ORIONE"/>
     <x v="0"/>
     <x v="1"/>
     <s v="R14 LOG"/>
@@ -2013,7 +2013,7 @@
     <row r="9" ht="14.4" customHeight="1">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Zona</t>
+          <t>Localidad</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2161,9 +2161,8 @@
   <dimension ref="A1:AF3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col width="11" customWidth="1" min="1" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="1" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
     <col width="19" customWidth="1" min="10" max="10"/>
     <col width="11" customWidth="1" min="11" max="13"/>
     <col width="12" customWidth="1" min="14" max="16"/>
@@ -2207,27 +2206,27 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Zona</t>
+          <t>Localidad</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>Partido</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>Subzona</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Region UN</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Categoria UN</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Localidad</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
@@ -2370,22 +2369,22 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
+          <t>Lanus</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
           <t>Zona 4</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>SAE LANUS</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Zona 4</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>LANUS</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -2498,20 +2497,20 @@
           <t>DON ORIONE</t>
         </is>
       </c>
-      <c r="F3" s="2" t="n"/>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Almirante Brown</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="n"/>
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>SAE BROWN</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Don Orione</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>DON ORIONE</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">

</xml_diff>